<commit_message>
Projecten-sjabloon: kolom Adres toegevoegd
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XayoweC5i4oaWG3ZU3bfMX
</commit_message>
<xml_diff>
--- a/documenten/Alwiti projecten import sjabloon.xlsx
+++ b/documenten/Alwiti projecten import sjabloon.xlsx
@@ -429,12 +429,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="48" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
@@ -451,10 +451,15 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Adres</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>Plaats</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Urenbudget</t>
         </is>
@@ -473,10 +478,15 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>Stadswerven 12</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>Dordrecht</t>
         </is>
       </c>
-      <c r="D2" t="n">
+      <c r="E2" t="n">
         <v>400</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Urenbudget per project verdeeld in buiten, werkplaats en meerwerk
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XayoweC5i4oaWG3ZU3bfMX
</commit_message>
<xml_diff>
--- a/documenten/Alwiti projecten import sjabloon.xlsx
+++ b/documenten/Alwiti projecten import sjabloon.xlsx
@@ -429,13 +429,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="48" customWidth="1" min="2" max="2"/>
     <col width="26" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
+    <col width="19" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -461,6 +465,21 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Budget buiten</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Budget werkplaats</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Budget meerwerk</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Urenbudget</t>
         </is>
       </c>
@@ -487,7 +506,13 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>400</v>
+        <v>300</v>
+      </c>
+      <c r="F2" t="n">
+        <v>80</v>
+      </c>
+      <c r="G2" t="n">
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -501,7 +526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="95" customWidth="1" min="1" max="1"/>
@@ -517,7 +542,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Projectnummer en Naam zijn verplicht, Plaats en Urenbudget mogen leeg.</t>
+          <t>Projectnummer en Naam zijn verplicht. Adres, Plaats en de budgetten mogen leeg.</t>
         </is>
       </c>
     </row>
@@ -546,6 +571,27 @@
       <c r="A6" t="inlineStr">
         <is>
           <t>Importeren: app → Projecten → Projecten importeren uit Excel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Budget buiten, werkplaats en meerwerk: uren per onderdeel. Het totaal wordt dan automatisch de som.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Meerwerk = uren die de monteur invult met type Meerwerk. Buiten en werkplaats zijn de overige uren op de bouw of in de werkplaats.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Urenbudget: alleen invullen als je het budget niet verdeelt (één totaal).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Uren tot nu toe per project in één keer invoeren
Kantoor kan per project de uren invullen die al gemaakt zijn maar niet in de app
staan (buiten/werkplaats/meerwerk, t/m datum). Ze tellen mee in urenbudget,
budgetgrafiek, Excel-export en het tabblad Werken van de Sheet. Ook via de
Excel-import (kolommen Tot nu toe buiten/werkplaats/meerwerk).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DwmETRLxA9tFxkzMRtNA8y
</commit_message>
<xml_diff>
--- a/documenten/Alwiti projecten import sjabloon.xlsx
+++ b/documenten/Alwiti projecten import sjabloon.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -440,6 +440,9 @@
     <col width="21" customWidth="1" min="6" max="6"/>
     <col width="19" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -481,6 +484,21 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Urenbudget</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Tot nu toe buiten</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Tot nu toe werkplaats</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Tot nu toe meerwerk</t>
         </is>
       </c>
     </row>

</xml_diff>